<commit_message>
Store and show only masked personal data
Names, NIK and addresses are now generated and stored already masked
(Budi W*****, 3273********0002, Jl. M****** No. **), and customer emails
no longer contain names (customer.0001@gmail.example). NIK in file names
is detected in masked form; the DP-11 scan now fails on any unmasked,
valid-looking NIK. Test fixtures use the same masked format.
Data, letters, reports, deck and case study regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RcpasmBE1hvgdead6uZREF
</commit_message>
<xml_diff>
--- a/reports/monthly_control_report.xlsx
+++ b/reports/monthly_control_report.xlsx
@@ -589,19 +589,19 @@
         <v>150</v>
       </c>
       <c r="F2" t="n">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="G2" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H2" t="n">
         <v>1</v>
       </c>
       <c r="I2" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="J2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -610,10 +610,10 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
@@ -622,13 +622,13 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="R2" t="n">
         <v>5</v>
       </c>
       <c r="S2" t="n">
-        <v>13.6</v>
+        <v>12.4</v>
       </c>
       <c r="T2" t="n">
         <v>10</v>
@@ -662,19 +662,19 @@
         <v>150</v>
       </c>
       <c r="F3" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="G3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
       </c>
       <c r="I3" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.08</v>
       </c>
       <c r="J3" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -683,10 +683,10 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="N3" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -695,13 +695,13 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>11.6</v>
+        <v>13.1</v>
       </c>
       <c r="T3" t="n">
         <v>10</v>
@@ -735,19 +735,19 @@
         <v>150</v>
       </c>
       <c r="F4" t="n">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>0.0867</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="J4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -756,10 +756,10 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O4" t="n">
         <v>0</v>
@@ -768,13 +768,13 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="R4" t="n">
         <v>2</v>
       </c>
       <c r="S4" t="n">
-        <v>12.1</v>
+        <v>12.8</v>
       </c>
       <c r="T4" t="n">
         <v>10</v>
@@ -849,10 +849,10 @@
         </is>
       </c>
       <c r="C2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" t="n">
         <v>1</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
       </c>
       <c r="E2" t="n">
         <v>2</v>
@@ -927,7 +927,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
@@ -979,13 +979,13 @@
         </is>
       </c>
       <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
         <v>2</v>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>3</v>
-      </c>
-      <c r="E7" t="n">
-        <v>2</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1120,13 +1120,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -1136,13 +1136,13 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="n">
-        <v>4</v>
-      </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -1152,10 +1152,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
@@ -1168,13 +1168,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1184,13 +1184,13 @@
         </is>
       </c>
       <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
         <v>2</v>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -1200,13 +1200,13 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
         <v>1</v>
       </c>
-      <c r="C7" t="n">
-        <v>4</v>
-      </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1220,7 +1220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1229,7 +1229,7 @@
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="56" customWidth="1" min="7" max="7"/>
+    <col width="59" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="59" customWidth="1" min="10" max="10"/>
@@ -1307,27 +1307,32 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7751182194</t>
+          <t>7748747227</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MDN</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>l***@outlook.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>branch.mdn@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT_7748747227_202608.pdf</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1337,22 +1342,22 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>DP-01</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Every customer on the send list has a letter</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>No letter found for this customer</t>
+          <t>Send-list email c***@gmial.example differs from master c***@gmail.example</t>
         </is>
       </c>
     </row>
@@ -1364,32 +1369,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7779425041</t>
+          <t>7748747227</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>MDN</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>a***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>branch.mdn@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7779425041_202608.pdf</t>
+          <t>REINSTATEMENT_7748747227_202608.pdf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1414,7 +1419,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Send-list email a***@gmail.example differs from master a***@gmail.example</t>
+          <t>Email domain looks like a typo of gmail.example</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1431,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7745671728</t>
+          <t>7744558470</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1436,22 +1441,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SBY</t>
+          <t>JKT</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>i***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.jkt@nusantaralife.example</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7745671728_202608.pdf</t>
+          <t>REINSTATEMENT_7744558470_202608.pdf</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1476,7 +1481,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Letter shows policy 7732055405 instead of 7745671728</t>
+          <t>NIK in letter (7315********5785) does not belong to recipient</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1493,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7745671728</t>
+          <t>7754915463</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1498,22 +1503,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SBY</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>i***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7745671728_202608.pdf</t>
+          <t>REINSTATEMENT_7754915463_202608.pdf</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1538,7 +1543,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Policyholder name in letter does not match recipient</t>
+          <t>Letter shows policy 7719031847 instead of 7754915463</t>
         </is>
       </c>
     </row>
@@ -1550,7 +1555,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7745671728</t>
+          <t>7754915463</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1560,22 +1565,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SBY</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>i***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7745671728_202608.pdf</t>
+          <t>REINSTATEMENT_7754915463_202608.pdf</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1600,7 +1605,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>NIK in letter (3228********7715) does not belong to recipient</t>
+          <t>Policyholder name in letter does not match recipient</t>
         </is>
       </c>
     </row>
@@ -1612,32 +1617,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>7756144614</t>
+          <t>7754915463</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>g***@outlook.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7756144614_202608.pdf</t>
+          <t>REINSTATEMENT_7754915463_202608.pdf</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1662,7 +1667,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>NIK in letter (1216********9215) does not belong to recipient</t>
+          <t>NIK in letter (3205********9580) does not belong to recipient</t>
         </is>
       </c>
     </row>
@@ -1674,27 +1679,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>7749826421</t>
+          <t>7786284849</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>MATURITY</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>SBY</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>MATURITY_7749826421_202608.pdf</t>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1704,22 +1709,22 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>DP-08</t>
+          <t>DP-01</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>One email = one customer + their own branch, no BCC</t>
+          <t>Every customer on the send list has a letter</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Email field holds more than one / an invalid address</t>
+          <t>No letter found for this customer</t>
         </is>
       </c>
     </row>
@@ -1731,27 +1736,32 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>7768739957</t>
+          <t>7788035038</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>MATURITY</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>n***@yahoo.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>MATURITY_7788035038_202608.pdf</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1761,22 +1771,22 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>DP-02</t>
+          <t>DP-07</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>No duplicate letters for one customer</t>
+          <t>Branch CC resolved from branch master and allowlisted</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2 letters found: BENEFIT_PAYMENT_7768739957_202608.pdf, BENEFIT_PAYMENT_7768739957_202608_revised.pdf</t>
+          <t>Manual CC y***@gmail.example is not the customer's branch mailbox</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1798,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>7702539622</t>
+          <t>7775513957</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1798,22 +1808,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>SBY</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>a***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>branch.bdg@nusantaralife.example</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>REINSTATEMENT_7702539622_202608.pdf</t>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1823,22 +1828,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-01</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>Every customer on the send list has a letter</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Send-list email a***@gmial.example differs from master a***@gmail.example</t>
+          <t>No letter found for this customer</t>
         </is>
       </c>
     </row>
@@ -1850,32 +1855,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>7702539622</t>
+          <t>7719457637</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>JKT</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>a***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>branch.bdg@nusantaralife.example</t>
+          <t>branch.jkt@nusantaralife.example</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7702539622_202608.pdf</t>
+          <t>BENEFIT_PAYMENT_7719457637_NIK3108xxxxxxxx4214_202608.pdf</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1885,22 +1890,22 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-10</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>NIK never appears in file name, subject or email body</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Email domain looks like a typo of gmail.example</t>
+          <t>File name contains a NIK</t>
         </is>
       </c>
     </row>
@@ -1912,7 +1917,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>7735920520</t>
+          <t>7762652962</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1922,22 +1927,17 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>SBY</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>j***@outlook.example</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7735920520_3512********0042_202608.pdf</t>
+          <t>BENEFIT_PAYMENT_7762652962_202608.pdf</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1947,22 +1947,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>DP-10</t>
+          <t>DP-08</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>NIK never appears in file name, subject or email body</t>
+          <t>One email = one customer + their own branch, no BCC</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>File name contains a 16-digit NIK</t>
+          <t>Email field holds more than one / an invalid address</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>7709842400</t>
+          <t>7709444919</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1984,22 +1984,17 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>l***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>MATURITY_7709842400_202608.pdf</t>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2009,22 +2004,22 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>DP-07</t>
+          <t>DP-03</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Branch CC resolved from branch master and allowlisted</t>
+          <t>File name points to exactly one policy</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Manual CC m***@gmail.example is not the customer's branch mailbox</t>
+          <t>Referenced by ambiguous file name(s): MATURITY_7709444919_REF7793838542_202608.pdf</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2031,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>7760486169</t>
+          <t>7793838542</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2046,22 +2041,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MDN</t>
+          <t>JKT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>l***@gmail.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>branch.mdn@nusantaralife.example</t>
+          <t>branch.jkt@nusantaralife.example</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7760486169_202608.pdf</t>
+          <t>REINSTATEMENT_7793838542_202608.pdf</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2071,22 +2066,22 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>DP-07</t>
+          <t>DP-03</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Branch CC resolved from branch master and allowlisted</t>
+          <t>File name points to exactly one policy</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Send-list branch JKT differs from master branch MDN</t>
+          <t>Referenced by ambiguous file name(s): MATURITY_7709444919_REF7793838542_202608.pdf</t>
         </is>
       </c>
     </row>
@@ -2098,32 +2093,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7706342956</t>
+          <t>7792504463</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MATURITY</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>JKT</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>g***@outlook.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>branch.jkt@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>MATURITY_7706342956_202608.pdf</t>
+          <t>BENEFIT_PAYMENT_7792504463_202608.pdf</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2133,22 +2128,22 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>DP-03</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>File name points to exactly one policy</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Referenced by ambiguous file name(s): MATURITY_7763303355_REF7706342956_202608.pdf</t>
+          <t>Send-list email c***@yahoo.example differs from master c***@yahoo.example</t>
         </is>
       </c>
     </row>
@@ -2160,7 +2155,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>7763303355</t>
+          <t>7778175903</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2175,7 +2170,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>v***@yahoo.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2190,12 +2185,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>DP-03</t>
+          <t>DP-02</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>File name points to exactly one policy</t>
+          <t>No duplicate letters for one customer</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -2205,7 +2200,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Referenced by ambiguous file name(s): MATURITY_7763303355_REF7706342956_202608.pdf</t>
+          <t>2 letters found: MATURITY_7778175903_202608.pdf, MATURITY_7778175903_202608_revised.pdf</t>
         </is>
       </c>
     </row>
@@ -2217,12 +2212,32 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>7742432766</t>
+          <t>7764643598</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BENEFIT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SBY</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>c***@gmail.example</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>MATURITY_7742432766_202608.pdf</t>
+          <t>BENEFIT_PAYMENT_7764643598_202608.pdf</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2232,54 +2247,59 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>DP-05</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>No orphan letter without an owner on the send list</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Letter has no owner on this send list - held, never sent</t>
+          <t>Send-list email c***@gmail.example differs from master c***@gmail.example</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>7754432040</t>
+          <t>7718481308</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>MATURITY</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>JKT</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>e***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.jkt@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>MATURITY_7718481308_202608.pdf</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2289,39 +2309,39 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DP-01</t>
+          <t>DP-07</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Every customer on the send list has a letter</t>
+          <t>Branch CC resolved from branch master and allowlisted</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>No letter found for this customer</t>
+          <t>Send-list branch BDG differs from master branch JKT</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7701559388</t>
+          <t>7720403813</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2331,7 +2351,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>a***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2339,6 +2359,11 @@
           <t>branch.ygy@nusantaralife.example</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>BENEFIT_PAYMENT_7720403813_202608.pdf</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>QUARANTINE</t>
@@ -2346,34 +2371,34 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>DP-02</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>No duplicate letters for one customer</t>
+          <t>Letter content (policy, name, NIK) matches the recipient</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2 letters found: REINSTATEMENT_7701559388_202609.pdf, REINSTATEMENT_7701559388_202609_revised.pdf</t>
+          <t>Letter shows policy 7792070437 instead of 7720403813</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>7717262909</t>
+          <t>7720403813</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2383,17 +2408,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>JKT</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>h***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>branch.jkt@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>BENEFIT_PAYMENT_7720403813_202608.pdf</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2403,59 +2433,59 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>DP-03</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>File name points to exactly one policy</t>
+          <t>Letter content (policy, name, NIK) matches the recipient</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Referenced by ambiguous file name(s): BENEFIT_PAYMENT_7717262909_REF7700813433_202609.pdf</t>
+          <t>Policyholder name in letter does not match recipient</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>7751164647</t>
+          <t>7720403813</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MATURITY</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>p***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>branch.bdg@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>MATURITY_7751164647_202609.pdf</t>
+          <t>BENEFIT_PAYMENT_7720403813_202608.pdf</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2465,12 +2495,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>Letter content (policy, name, NIK) matches the recipient</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2480,44 +2510,24 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Send-list email p***@gmial.example differs from master p***@gmail.example</t>
+          <t>NIK in letter (1226********8514) does not belong to recipient</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>7751164647</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>MATURITY</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>BDG</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>p***@gmail.example</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>branch.bdg@nusantaralife.example</t>
+          <t>7700846238</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>MATURITY_7751164647_202609.pdf</t>
+          <t>MATURITY_7700846238_202608.pdf</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2527,22 +2537,22 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-05</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>No orphan letter without an owner on the send list</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Email domain looks like a typo of gmail.example</t>
+          <t>Letter has no owner on this send list - held, never sent</t>
         </is>
       </c>
     </row>
@@ -2554,32 +2564,32 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>7710321322</t>
+          <t>7773965956</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>MATURITY</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>YGY</t>
+          <t>SBY</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>e***@gmail.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>branch.ygy@nusantaralife.example</t>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7710321322_202609.pdf</t>
+          <t>MATURITY_7773965956_NIK3518xxxxxxxx9007_202609.pdf</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2589,22 +2599,22 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-10</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>NIK never appears in file name, subject or email body</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Send-list email e***@gmail.example differs from master e***@gmail.example</t>
+          <t>File name contains a NIK</t>
         </is>
       </c>
     </row>
@@ -2616,32 +2626,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>7727221816</t>
+          <t>7789264626</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>MATURITY</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>MDN</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>r***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>branch.mdn@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7727221816_202609.pdf</t>
+          <t>MATURITY_7789264626_202609.pdf</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2666,7 +2676,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>NIK in letter (3204********0420) does not belong to recipient</t>
+          <t>NIK in letter (3224********1546) does not belong to recipient</t>
         </is>
       </c>
     </row>
@@ -2678,7 +2688,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>7700813433</t>
+          <t>7700233103</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2688,22 +2698,17 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>JKT</t>
+          <t>SBY</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>g***@outlook.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>branch.jkt@nusantaralife.example</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>MATURITY_7700813433_202609.pdf</t>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2713,12 +2718,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>DP-03</t>
+          <t>DP-01</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>File name points to exactly one policy</t>
+          <t>Every customer on the send list has a letter</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -2728,7 +2733,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Referenced by ambiguous file name(s): BENEFIT_PAYMENT_7717262909_REF7700813433_202609.pdf</t>
+          <t>No letter found for this customer</t>
         </is>
       </c>
     </row>
@@ -2740,12 +2745,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>7721151267</t>
+          <t>7704917079</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2753,11 +2758,6 @@
           <t>JKT</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>m***@outlook.example</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>branch.jkt@nusantaralife.example</t>
@@ -2765,7 +2765,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7721151267_202609.pdf</t>
+          <t>BENEFIT_PAYMENT_7704917079_202609.pdf</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2775,12 +2775,12 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>DP-07</t>
+          <t>DP-08</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Branch CC resolved from branch master and allowlisted</t>
+          <t>One email = one customer + their own branch, no BCC</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Manual CC j***@gmail.example is not the customer's branch mailbox</t>
+          <t>Email field holds more than one / an invalid address</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2802,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>7750165584</t>
+          <t>7787171057</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2817,7 +2817,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>y***@outlook.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2827,7 +2827,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7750165584_3213********9671_202609.pdf</t>
+          <t>REINSTATEMENT_7787171057_202609.pdf</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2837,22 +2837,22 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>DP-10</t>
+          <t>DP-07</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>NIK never appears in file name, subject or email body</t>
+          <t>Branch CC resolved from branch master and allowlisted</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>File name contains a 16-digit NIK</t>
+          <t>Manual CC b***@gmail.example is not the customer's branch mailbox</t>
         </is>
       </c>
     </row>
@@ -2864,32 +2864,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>7783839028</t>
+          <t>7781089846</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>YGY</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>u***@yahoo.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>branch.ygy@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7783839028_202609.pdf</t>
+          <t>REINSTATEMENT_7781089846_202609.pdf</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2899,12 +2899,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-07</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>Branch CC resolved from branch master and allowlisted</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Send-list email u***@yahoo.example differs from master u***@yahoo.example</t>
+          <t>Send-list branch JKT differs from master branch BDG</t>
         </is>
       </c>
     </row>
@@ -2926,27 +2926,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>7706342956</t>
+          <t>7715126130</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>MATURITY</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>JKT</t>
+          <t>SBY</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>branch.jkt@nusantaralife.example</t>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>MATURITY_7706342956_202609.pdf</t>
+          <t>BENEFIT_PAYMENT_7715126130_202609.pdf</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2956,12 +2961,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>DP-08</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>One email = one customer + their own branch, no BCC</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2971,7 +2976,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Email field holds more than one / an invalid address</t>
+          <t>Send-list email c***@gmail.example differs from master c***@gmail.example</t>
         </is>
       </c>
     </row>
@@ -2983,7 +2988,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>7757426050</t>
+          <t>7725955055</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2993,22 +2998,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>o***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7757426050_202609.pdf</t>
+          <t>BENEFIT_PAYMENT_7725955055_202609.pdf</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3033,7 +3038,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Letter shows policy 7794744011 instead of 7757426050</t>
+          <t>Letter shows policy 7761678333 instead of 7725955055</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3050,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>7757426050</t>
+          <t>7725955055</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3055,22 +3060,22 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>o***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7757426050_202609.pdf</t>
+          <t>BENEFIT_PAYMENT_7725955055_202609.pdf</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -3107,7 +3112,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>7757426050</t>
+          <t>7725955055</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3117,22 +3122,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>o***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7757426050_202609.pdf</t>
+          <t>BENEFIT_PAYMENT_7725955055_202609.pdf</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3157,7 +3162,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>NIK in letter (3210********3283) does not belong to recipient</t>
+          <t>NIK in letter (7311********3378) does not belong to recipient</t>
         </is>
       </c>
     </row>
@@ -3169,27 +3174,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>7796323595</t>
+          <t>7743335070</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>MATURITY</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>YGY</t>
+          <t>MKS</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>p***@outlook.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>branch.ygy@nusantaralife.example</t>
+          <t>branch.mks@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT_7743335070_202609.pdf</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -3199,22 +3209,22 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>DP-01</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Every customer on the send list has a letter</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>No letter found for this customer</t>
+          <t>Send-list email c***@gmial.example differs from master c***@gmail.example</t>
         </is>
       </c>
     </row>
@@ -3226,32 +3236,32 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>7736781978</t>
+          <t>7743335070</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MATURITY</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SBY</t>
+          <t>MKS</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>w***@yahoo.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.mks@nusantaralife.example</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>MATURITY_7736781978_202609.pdf</t>
+          <t>REINSTATEMENT_7743335070_202609.pdf</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -3261,12 +3271,12 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>DP-07</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Branch CC resolved from branch master and allowlisted</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -3276,7 +3286,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Send-list branch JKT differs from master branch SBY</t>
+          <t>Email domain looks like a typo of gmail.example</t>
         </is>
       </c>
     </row>
@@ -3288,12 +3298,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>7740467843</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>MATURITY_7740467843_202609.pdf</t>
+          <t>7714090496</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>MDN</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>c***@gmail.example</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -3303,12 +3328,12 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>DP-05</t>
+          <t>DP-03</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>No orphan letter without an owner on the send list</t>
+          <t>File name points to exactly one policy</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -3318,44 +3343,39 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Letter has no owner on this send list - held, never sent</t>
+          <t>Referenced by ambiguous file name(s): REINSTATEMENT_7714090496_REF7716650857_202609.pdf</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>7783839028</t>
+          <t>7760787811</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>BENEFIT_PAYMENT</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>YGY</t>
+          <t>SBY</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>u***@yahoo.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>branch.ygy@nusantaralife.example</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>REINSTATEMENT_7783839028_202610.pdf</t>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3365,34 +3385,34 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-02</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>No duplicate letters for one customer</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Send-list email u***@gmial.example differs from master u***@yahoo.example</t>
+          <t>2 letters found: BENEFIT_PAYMENT_7760787811_202609.pdf, BENEFIT_PAYMENT_7760787811_202609_revised.pdf</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>7783839028</t>
+          <t>7716650857</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -3402,22 +3422,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>YGY</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>u***@yahoo.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>branch.ygy@nusantaralife.example</t>
+          <t>branch.bdg@nusantaralife.example</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>REINSTATEMENT_7783839028_202610.pdf</t>
+          <t>REINSTATEMENT_7716650857_202609.pdf</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3427,59 +3447,39 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-03</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>File name points to exactly one policy</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Email domain looks like a typo of gmail.example</t>
+          <t>Referenced by ambiguous file name(s): REINSTATEMENT_7714090496_REF7716650857_202609.pdf</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>7785989243</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>MATURITY</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>MDN</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>y***@gmail.example</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>branch.mdn@nusantaralife.example</t>
+          <t>7788296150</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>MATURITY_7785989243_202610.pdf</t>
+          <t>MATURITY_7788296150_202609.pdf</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3489,22 +3489,22 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>DP-06</t>
+          <t>DP-05</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Customer email matches master data and has no domain typo</t>
+          <t>No orphan letter without an owner on the send list</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Send-list email y***@gmail.example differs from master y***@gmail.example</t>
+          <t>Letter has no owner on this send list - held, never sent</t>
         </is>
       </c>
     </row>
@@ -3516,27 +3516,32 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>7736781978</t>
+          <t>7722463353</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SBY</t>
+          <t>MDN</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7736781978_202610.pdf</t>
+          <t>REINSTATEMENT_7722463353_202610.pdf</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3546,12 +3551,12 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>DP-08</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>One email = one customer + their own branch, no BCC</t>
+          <t>Letter content (policy, name, NIK) matches the recipient</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -3561,7 +3566,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Email field holds more than one / an invalid address</t>
+          <t>Letter shows policy 7731273768 instead of 7722463353</t>
         </is>
       </c>
     </row>
@@ -3573,32 +3578,32 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>7755885086</t>
+          <t>7722463353</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>w***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>branch.bdg@nusantaralife.example</t>
+          <t>branch.mdn@nusantaralife.example</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7755885086_202610.pdf</t>
+          <t>REINSTATEMENT_7722463353_202610.pdf</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3608,12 +3613,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>DP-07</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Branch CC resolved from branch master and allowlisted</t>
+          <t>Letter content (policy, name, NIK) matches the recipient</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3623,7 +3628,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Manual CC b***@gmail.example is not the customer's branch mailbox</t>
+          <t>Policyholder name in letter does not match recipient</t>
         </is>
       </c>
     </row>
@@ -3635,27 +3640,32 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>7792660933</t>
+          <t>7722463353</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MATURITY</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>a***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.mdn@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT_7722463353_202610.pdf</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3665,22 +3675,22 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>DP-03</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>File name points to exactly one policy</t>
+          <t>Letter content (policy, name, NIK) matches the recipient</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Referenced by ambiguous file name(s): MATURITY_7792660933_REF7712316065_202610.pdf</t>
+          <t>NIK in letter (3420********6607) does not belong to recipient</t>
         </is>
       </c>
     </row>
@@ -3692,12 +3702,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>7712316065</t>
+          <t>7776524680</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -3707,7 +3717,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>y***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3717,7 +3727,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7712316065_202610.pdf</t>
+          <t>REINSTATEMENT_7776524680_202610.pdf</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
@@ -3727,22 +3737,22 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>DP-03</t>
+          <t>DP-07</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>File name points to exactly one policy</t>
+          <t>Branch CC resolved from branch master and allowlisted</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Referenced by ambiguous file name(s): MATURITY_7792660933_REF7712316065_202610.pdf</t>
+          <t>Manual CC y***@gmail.example is not the customer's branch mailbox</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3764,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>7741716988</t>
+          <t>7725189553</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -3764,22 +3774,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>MKS</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>l***@outlook.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>branch.bdg@nusantaralife.example</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>MATURITY_7741716988_202610.pdf</t>
+          <t>branch.mks@nusantaralife.example</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -3789,22 +3794,22 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>DP-04</t>
+          <t>DP-01</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Letter content (policy, name, NIK) matches the recipient</t>
+          <t>Every customer on the send list has a letter</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Letter shows policy 7721151267 instead of 7741716988</t>
+          <t>No letter found for this customer</t>
         </is>
       </c>
     </row>
@@ -3816,7 +3821,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>7741716988</t>
+          <t>7779501978</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -3826,22 +3831,22 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>l***@outlook.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>branch.bdg@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>MATURITY_7741716988_202610.pdf</t>
+          <t>MATURITY_7779501978_202610.pdf</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -3851,12 +3856,12 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>DP-04</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Letter content (policy, name, NIK) matches the recipient</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -3866,7 +3871,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Policyholder name in letter does not match recipient</t>
+          <t>Send-list email c***@gmial.example differs from master c***@outlook.example</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3883,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>7741716988</t>
+          <t>7779501978</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -3888,22 +3893,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>l***@outlook.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>branch.bdg@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>MATURITY_7741716988_202610.pdf</t>
+          <t>MATURITY_7779501978_202610.pdf</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3913,12 +3918,12 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>DP-04</t>
+          <t>DP-06</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Letter content (policy, name, NIK) matches the recipient</t>
+          <t>Customer email matches master data and has no domain typo</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -3928,7 +3933,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>NIK in letter (3122********6393) does not belong to recipient</t>
+          <t>Email domain looks like a typo of gmail.example</t>
         </is>
       </c>
     </row>
@@ -3940,32 +3945,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>7788089448</t>
+          <t>7775513957</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>MDN</t>
+          <t>SBY</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>m***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>branch.mdn@nusantaralife.example</t>
+          <t>branch.sby@nusantaralife.example</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7788089448_202610.pdf</t>
+          <t>REINSTATEMENT_7775513957_202610.pdf</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -3975,22 +3980,22 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>DP-04</t>
+          <t>DP-03</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Letter content (policy, name, NIK) matches the recipient</t>
+          <t>File name points to exactly one policy</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>CRITICAL</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>NIK in letter (3224********6732) does not belong to recipient</t>
+          <t>Referenced by ambiguous file name(s): BENEFIT_PAYMENT_7759130138_REF7775513957_202610.pdf</t>
         </is>
       </c>
     </row>
@@ -4002,32 +4007,32 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>7755849998</t>
+          <t>7756602216</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>SBY</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>o***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT_7755849998_202610.pdf</t>
+          <t>REINSTATEMENT_7756602216_202610.pdf</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -4037,12 +4042,12 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>DP-07</t>
+          <t>DP-04</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Branch CC resolved from branch master and allowlisted</t>
+          <t>Letter content (policy, name, NIK) matches the recipient</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -4052,7 +4057,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Send-list branch JKT differs from master branch SBY</t>
+          <t>NIK in letter (3415********5932) does not belong to recipient</t>
         </is>
       </c>
     </row>
@@ -4064,27 +4069,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>7714902427</t>
+          <t>7732561133</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BENEFIT_PAYMENT</t>
+          <t>REINSTATEMENT</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>MKS</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>w***@gmail.example</t>
+          <t>SBY</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.sby@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT_7732561133_202610.pdf</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -4094,22 +4099,22 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>DP-02</t>
+          <t>DP-08</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>No duplicate letters for one customer</t>
+          <t>One email = one customer + their own branch, no BCC</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>CRITICAL</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2 letters found: BENEFIT_PAYMENT_7714902427_202610.pdf, BENEFIT_PAYMENT_7714902427_202610_revised.pdf</t>
+          <t>Email field holds more than one / an invalid address</t>
         </is>
       </c>
     </row>
@@ -4121,27 +4126,27 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>7774895425</t>
+          <t>7775387892</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>MATURITY</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>MKS</t>
+          <t>JKT</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>y***@outlook.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>branch.mks@nusantaralife.example</t>
+          <t>branch.jkt@nusantaralife.example</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -4178,7 +4183,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>7705210085</t>
+          <t>7759130138</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -4188,22 +4193,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>YGY</t>
+          <t>JKT</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>e***@gmail.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>branch.ygy@nusantaralife.example</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>BENEFIT_PAYMENT_7705210085_3421********0744_202610.pdf</t>
+          <t>branch.jkt@nusantaralife.example</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -4213,12 +4213,12 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>DP-10</t>
+          <t>DP-03</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>NIK never appears in file name, subject or email body</t>
+          <t>File name points to exactly one policy</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>File name contains a 16-digit NIK</t>
+          <t>Referenced by ambiguous file name(s): BENEFIT_PAYMENT_7759130138_REF7775513957_202610.pdf</t>
         </is>
       </c>
     </row>
@@ -4240,27 +4240,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>7789676464</t>
+          <t>7722802311</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>REINSTATEMENT</t>
+          <t>MATURITY</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>SBY</t>
+          <t>YGY</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>i***@yahoo.example</t>
+          <t>c***@yahoo.example</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>branch.sby@nusantaralife.example</t>
+          <t>branch.ygy@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>MATURITY_7722802311_NIK3418xxxxxxxx3981_202610.pdf</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -4270,12 +4275,12 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>DP-01</t>
+          <t>DP-10</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Every customer on the send list has a letter</t>
+          <t>NIK never appears in file name, subject or email body</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -4285,7 +4290,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>No letter found for this customer</t>
+          <t>File name contains a NIK</t>
         </is>
       </c>
     </row>
@@ -4297,12 +4302,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>7718087769</t>
+          <t>7718627072</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>MATURITY</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>YGY</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>c***@gmail.example</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>branch.ygy@nusantaralife.example</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>MATURITY_7718087769_202610.pdf</t>
+          <t>MATURITY_7718627072_202610.pdf</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -4312,20 +4337,243 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
+          <t>DP-06</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>Customer email matches master data and has no domain typo</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Send-list email c***@gmail.example differs from master c***@gmail.example</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>7728750039</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>YGY</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>c***@yahoo.example</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>branch.ygy@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT_7728750039_202610.pdf</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>DP-07</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>Branch CC resolved from branch master and allowlisted</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Send-list branch JKT differs from master branch YGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>7776698447</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>BENEFIT_PAYMENT</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>MDN</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>c***@outlook.example</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>branch.mdn@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>DP-02</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>No duplicate letters for one customer</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2 letters found: BENEFIT_PAYMENT_7776698447_202610.pdf, BENEFIT_PAYMENT_7776698447_202610_revised.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>7799119294</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>JKT</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>c***@gmail.example</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>branch.jkt@nusantaralife.example</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>REINSTATEMENT_7799119294_202610.pdf</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>DP-06</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>Customer email matches master data and has no domain typo</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Send-list email c***@gmail.example differs from master c***@gmail.example</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>7731009808</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>MATURITY_7731009808_202610.pdf</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>QUARANTINE</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
           <t>DP-05</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="J56" t="inlineStr">
         <is>
           <t>No orphan letter without an owner on the send list</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="L52" t="inlineStr">
+      <c r="L56" t="inlineStr">
         <is>
           <t>Letter has no owner on this send list - held, never sent</t>
         </is>
@@ -4398,7 +4646,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -4426,7 +4674,7 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>79</v>
+        <v>53</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
@@ -4454,7 +4702,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -4482,7 +4730,7 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -4510,7 +4758,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
@@ -4538,7 +4786,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>63</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -4609,7 +4857,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>7727134379</t>
+          <t>7744765114</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4619,7 +4867,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>n***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -4646,17 +4894,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>7725970383</t>
+          <t>7787171057</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>YGY</t>
+          <t>BDG</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>m***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4683,17 +4931,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7786214422</t>
+          <t>7777166781</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JKT</t>
+          <t>MDN</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>e***@outlook.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4720,7 +4968,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>7763643347</t>
+          <t>7708477974</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4730,7 +4978,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>t***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4757,17 +5005,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>7788942088</t>
+          <t>7709655248</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MDN</t>
+          <t>MKS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>d***@gmail.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4794,17 +5042,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>7757844933</t>
+          <t>7722623610</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>MKS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>s***@yahoo.example</t>
+          <t>c***@gmail.example</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4831,17 +5079,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>7719229864</t>
+          <t>7702768399</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BDG</t>
+          <t>JKT</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>m***@gmail.example</t>
+          <t>c***@outlook.example</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4929,7 +5177,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:04+00:00</t>
+          <t>2026-10-17T15:28:00+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4954,14 +5202,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>138 emails submitted for approval</t>
+          <t>135 emails submitted for approval</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:04+00:00</t>
+          <t>2026-10-17T15:28:00+00:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -4993,7 +5241,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:05+00:00</t>
+          <t>2026-10-17T15:28:01+00:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5018,14 +5266,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>138 emails sent, 0 transport errors</t>
+          <t>135 emails sent, 0 transport errors</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:16+00:00</t>
+          <t>2026-10-17T15:28:14+00:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5050,14 +5298,14 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>136 emails submitted for approval</t>
+          <t>138 emails submitted for approval</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:16+00:00</t>
+          <t>2026-10-17T15:28:14+00:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5089,7 +5337,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:17+00:00</t>
+          <t>2026-10-17T15:28:15+00:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5114,14 +5362,14 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>136 emails sent, 0 transport errors</t>
+          <t>138 emails sent, 0 transport errors</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:28+00:00</t>
+          <t>2026-10-17T15:28:27+00:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5146,14 +5394,14 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>137 emails submitted for approval</t>
+          <t>136 emails submitted for approval</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:28+00:00</t>
+          <t>2026-10-17T15:28:27+00:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5185,7 +5433,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-17T15:20:29+00:00</t>
+          <t>2026-10-17T15:28:28+00:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5210,7 +5458,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>137 emails sent, 0 transport errors</t>
+          <t>136 emails sent, 0 transport errors</t>
         </is>
       </c>
     </row>

</xml_diff>